<commit_message>
fixed bug of button lampiran
</commit_message>
<xml_diff>
--- a/assets/templates/Template_Data_Barang.xlsx
+++ b/assets/templates/Template_Data_Barang.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tegar\Downloads\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tegar\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C558D5AB-2F40-4C44-80F2-83C81FEB3D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFB40972-195F-4B63-B930-9525AB3AEA91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,13 +16,14 @@
     <sheet name="Template Data Barang" sheetId="1" r:id="rId1"/>
     <sheet name="Size" sheetId="2" r:id="rId2"/>
     <sheet name="Satuan" sheetId="3" r:id="rId3"/>
+    <sheet name="Kategori" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>No</t>
   </si>
@@ -115,6 +116,18 @@
   </si>
   <si>
     <t>BOX</t>
+  </si>
+  <si>
+    <t>Kategori</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Barang X</t>
+  </si>
+  <si>
+    <t>Special Price</t>
   </si>
 </sst>
 </file>
@@ -391,13 +404,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:N1000"/>
+  <dimension ref="A1:O1000"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="8" max="14" width="12.6640625" style="6"/>
+    <col min="1" max="1" width="5.109375" customWidth="1"/>
+    <col min="2" max="7" width="14.33203125" customWidth="1"/>
+    <col min="8" max="14" width="14.33203125" style="6" customWidth="1"/>
+    <col min="15" max="15" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -419,29 +435,32 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -457,7 +476,7 @@
       <c r="M2" s="5"/>
       <c r="N2" s="5"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -466,43 +485,43 @@
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
@@ -3461,7 +3480,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F718C934-FCA2-450F-A99A-1688DDC6FD8A}">
           <x14:formula1>
             <xm:f>Size!$A$1:$A$12</xm:f>
@@ -3473,6 +3492,12 @@
             <xm:f>Satuan!$A$1:$A$5</xm:f>
           </x14:formula1>
           <xm:sqref>F2:F1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A413F143-9DAF-4AA5-8E50-A2CD3B2598C5}">
+          <x14:formula1>
+            <xm:f>Kategori!$A$1:$A$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>H2:H1001</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3583,4 +3608,29 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEADA618-17DC-458E-B415-E04D6FACC83B}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Backup perubahan langsung dari Hostinger sebelum sync
</commit_message>
<xml_diff>
--- a/assets/templates/Template_Data_Barang.xlsx
+++ b/assets/templates/Template_Data_Barang.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tegar\Downloads\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tegar\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C558D5AB-2F40-4C44-80F2-83C81FEB3D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFB40972-195F-4B63-B930-9525AB3AEA91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,13 +16,14 @@
     <sheet name="Template Data Barang" sheetId="1" r:id="rId1"/>
     <sheet name="Size" sheetId="2" r:id="rId2"/>
     <sheet name="Satuan" sheetId="3" r:id="rId3"/>
+    <sheet name="Kategori" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>No</t>
   </si>
@@ -115,6 +116,18 @@
   </si>
   <si>
     <t>BOX</t>
+  </si>
+  <si>
+    <t>Kategori</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Barang X</t>
+  </si>
+  <si>
+    <t>Special Price</t>
   </si>
 </sst>
 </file>
@@ -391,13 +404,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:N1000"/>
+  <dimension ref="A1:O1000"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="8" max="14" width="12.6640625" style="6"/>
+    <col min="1" max="1" width="5.109375" customWidth="1"/>
+    <col min="2" max="7" width="14.33203125" customWidth="1"/>
+    <col min="8" max="14" width="14.33203125" style="6" customWidth="1"/>
+    <col min="15" max="15" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -419,29 +435,32 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -457,7 +476,7 @@
       <c r="M2" s="5"/>
       <c r="N2" s="5"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -466,43 +485,43 @@
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
@@ -3461,7 +3480,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F718C934-FCA2-450F-A99A-1688DDC6FD8A}">
           <x14:formula1>
             <xm:f>Size!$A$1:$A$12</xm:f>
@@ -3473,6 +3492,12 @@
             <xm:f>Satuan!$A$1:$A$5</xm:f>
           </x14:formula1>
           <xm:sqref>F2:F1001</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A413F143-9DAF-4AA5-8E50-A2CD3B2598C5}">
+          <x14:formula1>
+            <xm:f>Kategori!$A$1:$A$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>H2:H1001</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3583,4 +3608,29 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEADA618-17DC-458E-B415-E04D6FACC83B}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>